<commit_message>
new added in detection
</commit_message>
<xml_diff>
--- a/Detection/Detection paper link & details.xlsx
+++ b/Detection/Detection paper link & details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jihad\Skin-cancer-papers\Detection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAE7540B-3D4B-4915-992E-41CEB7C6E17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669EB7F5-63E6-46AA-8190-C24274CC3878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="57">
   <si>
     <t>Year</t>
   </si>
@@ -141,9 +141,6 @@
     <t>High-fidelity detection, subtyping, and localization of five skin neoplasms using supervised and semi-supervised learning</t>
   </si>
   <si>
-    <t>Supervised + Semi-supervised</t>
-  </si>
-  <si>
     <t>konta?</t>
   </si>
   <si>
@@ -163,13 +160,49 @@
   </si>
   <si>
     <t>Advancing skin cancer detection through deep learning and fusion of patient metadata and skin lesion images</t>
+  </si>
+  <si>
+    <t>Semi-supervised</t>
+  </si>
+  <si>
+    <t>Hypergraph-based contrastive embedding and attention fusion for detection of skin cancer</t>
+  </si>
+  <si>
+    <t>Multimodel mixed</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-026-43351-9</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S174680942600964X</t>
+  </si>
+  <si>
+    <t>XAAI-ledger: An explainable CNN-transformer-based multi-modal deep learning framework for early detection of melanoma and non-melanoma skin cancers using dermoscopic and clinical data</t>
+  </si>
+  <si>
+    <t>An Enhanced Skin Cancer Detection Method Utilizing TriBlendNet and Deepdilated Focus U-Net</t>
+  </si>
+  <si>
+    <t>https://www.etasr.com/index.php/ETASR/article/view/14192</t>
+  </si>
+  <si>
+    <t>Detection of multiclass non-melanoma skin cancer with multi-variable DCNN with hybrid gradient boosting optimizer</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S2090447925006975</t>
+  </si>
+  <si>
+    <t>Hybrid vision transformer and graph neural network model with region-adaptive attention for enhanced skin cancer prediction</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-025-32502-z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,13 +210,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -195,16 +242,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -495,7 +553,7 @@
   <sheetData>
     <row r="5" spans="4:9" x14ac:dyDescent="0.3">
       <c r="D5" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>0</v>
@@ -676,7 +734,7 @@
       <c r="F15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="H15" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I15" s="1" t="s">
@@ -724,17 +782,17 @@
       <c r="E18" s="1">
         <v>2022</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="19" spans="4:9" ht="115.2" x14ac:dyDescent="0.3">
@@ -745,13 +803,13 @@
         <v>2026</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>5</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="4:9" ht="100.8" x14ac:dyDescent="0.3">
@@ -762,38 +820,98 @@
         <v>2026</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>5</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21" spans="4:9" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="4:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="D21" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="22" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="E21" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="4:9" ht="172.8" x14ac:dyDescent="0.3">
       <c r="D22" s="1">
         <v>17</v>
       </c>
-    </row>
-    <row r="23" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="E22" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="4:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="D23" s="1">
         <v>18</v>
       </c>
-    </row>
-    <row r="24" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="E23" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="4:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="D24" s="1">
         <v>19</v>
       </c>
-    </row>
-    <row r="25" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="E24" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="4:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="D25" s="1">
         <v>20</v>
+      </c>
+      <c r="E25" s="1">
+        <v>2026</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="4:9" x14ac:dyDescent="0.3">
@@ -972,7 +1090,11 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H15" r:id="rId1" xr:uid="{1FC0EC8F-143F-4DE8-9A68-EAA020C3670D}"/>
+    <hyperlink ref="H18" r:id="rId2" xr:uid="{4EF12DB5-41F0-4EFF-8ADB-A95D44B803B9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
45 papers downloaded total
</commit_message>
<xml_diff>
--- a/Detection/Detection paper link & details.xlsx
+++ b/Detection/Detection paper link & details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jihad\Skin-cancer-papers\Detection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669EB7F5-63E6-46AA-8190-C24274CC3878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56CFFC8-E74C-4E2D-B208-6E18D9ADD9C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2616" yWindow="2616" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="61">
   <si>
     <t>Year</t>
   </si>
@@ -196,6 +196,18 @@
   </si>
   <si>
     <t>https://www.nature.com/articles/s41598-025-32502-z</t>
+  </si>
+  <si>
+    <t>Skin Cancer Detection using Machine Learning Classification Models</t>
+  </si>
+  <si>
+    <t>https://www.ijisae.org/index.php/IJISAE/article/view/3966/2616</t>
+  </si>
+  <si>
+    <t>Comparative analysis of multimodal architectures for effective skin lesion detection using clinical and image data</t>
+  </si>
+  <si>
+    <t>https://www.frontiersin.org/journals/artificial-intelligence/articles/10.3389/frai.2025.1608837/full?utm_source=chatgpt.com</t>
   </si>
 </sst>
 </file>
@@ -914,14 +926,38 @@
         <v>56</v>
       </c>
     </row>
-    <row r="26" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:9" ht="72" x14ac:dyDescent="0.3">
       <c r="D26" s="1">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="E26" s="1">
+        <v>2023</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="4:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="D27" s="1">
         <v>22</v>
+      </c>
+      <c r="E27" s="1">
+        <v>2025</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="4:9" x14ac:dyDescent="0.3">

</xml_diff>